<commit_message>
Add Exadata Cloud at Customer X11M BOM rules
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -567,7 +567,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Oracle Investment Proposal (as of 05/22/2026)</t>
+          <t>Oracle Investment Proposal (as of 06/22/2026)</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       <c r="A7"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Exadata Database Service</t>
+          <t>Exadata Database Service on Cloud@Customer X11M</t>
         </is>
       </c>
       <c r="C7"/>
@@ -690,7 +690,11 @@
       <c r="F7"/>
       <c r="G7"/>
       <c r="H7"/>
-      <c r="I7"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Test BOM baseline: single rack; High redundancy default; license model TBD - choose BYOL or License Included.</t>
+        </is>
+      </c>
       <c r="J7">
         <f>$K$3</f>
       </c>
@@ -702,33 +706,27 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>B110629</t>
-        </is>
-      </c>
+      <c r="A8"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Exadata Cloud Infrastructure - Storage Server - X11M (Hosted Environment Per Hour)</t>
+          <t>Exadata Cloud@Customer X11M Rack - single rack baseline</t>
         </is>
       </c>
       <c r="C8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
-      <c r="E8">
-        <v>744</v>
-      </c>
-      <c r="F8">
-        <v>2.9032</v>
-      </c>
-      <c r="G8">
-        <v>8639.9232</v>
-      </c>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
       <c r="H8"/>
-      <c r="I8"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Each rack should be modeled as prepopulated with 2 database servers.</t>
+        </is>
+      </c>
       <c r="J8">
         <f>$K$3</f>
       </c>
@@ -740,33 +738,27 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>B110627</t>
-        </is>
-      </c>
+      <c r="A9"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Exadata Cloud Infrastructure - Database Server - X11M (Hosted Environment Per Hour)</t>
+          <t>Exadata Database Service on Cloud@Customer X11M - Database Server</t>
         </is>
       </c>
       <c r="C9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
-      <c r="E9">
-        <v>744</v>
-      </c>
-      <c r="F9">
-        <v>2.9032</v>
-      </c>
-      <c r="G9">
-        <v>6479.9424</v>
-      </c>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
       <c r="H9"/>
-      <c r="I9"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Baseline single-rack configuration includes 2 database servers. Additional database servers increase usable memory and database cores/ECPUs.</t>
+        </is>
+      </c>
       <c r="J9">
         <f>$K$3</f>
       </c>
@@ -778,33 +770,27 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>B110631</t>
-        </is>
-      </c>
+      <c r="A10"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Exadata Database ECPU - Dedicated Infrastructure (ECPU Per Hour)</t>
+          <t>Exadata Database Service on Cloud@Customer X11M - Storage Server</t>
         </is>
       </c>
       <c r="C10">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
-      <c r="E10">
-        <v>744</v>
-      </c>
-      <c r="F10">
-        <v>0.336</v>
-      </c>
-      <c r="G10">
-        <v>5999.616</v>
-      </c>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10"/>
       <c r="H10"/>
-      <c r="I10"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Minimum storage-server count is 3. Assumes High redundancy unless Normal redundancy is explicitly specified.</t>
+        </is>
+      </c>
       <c r="J10">
         <f>$K$3</f>
       </c>
@@ -816,40 +802,72 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Monthly Total</t>
-        </is>
-      </c>
-      <c r="G11">
-        <f>SUM(G7:G10)</f>
+          <t>Exadata Database ECPU - Dedicated Infrastructure</t>
+        </is>
+      </c>
+      <c r="C11"/>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>744</v>
+      </c>
+      <c r="F11"/>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Software license model TBD - choose BYOL or License Included before final pricing.</t>
+        </is>
       </c>
       <c r="J11">
         <f>$K$3</f>
       </c>
       <c r="K11">
-        <f>SUM(K7:K10)</f>
+        <f>IF(G11="","",G11*(1-$K$3))</f>
       </c>
       <c r="L11">
-        <f>SUM(L7:L10)</f>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+        <f>IF(K11="","",K11*12)</f>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Monthly Total</t>
+        </is>
+      </c>
+      <c r="G12">
+        <f>SUM(G7:G11)</f>
+      </c>
+      <c r="J12">
+        <f>$K$3</f>
+      </c>
+      <c r="K12">
+        <f>SUM(K7:K11)</f>
+      </c>
+      <c r="L12">
+        <f>SUM(L7:L11)</f>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Quote is for investment proposal only.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Disclaimer: Pricing is an estimate based on Oracle Cost Estimator or user-provided list-price inputs. It is not a formal Oracle quote. Validate pricing, terms, discounts, and availability with Oracle before procurement.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:L11"/>
+  <autoFilter ref="A6:L12"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update BOM workbook calculations and docs
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -6,7 +6,7 @@
   <sheets>
     <sheet sheetId="1" name="PAAS" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -95,6 +95,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -146,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -200,6 +203,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -547,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -558,16 +562,16 @@
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="28" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="12" max="12" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Oracle Investment Proposal (as of 06/22/2026)</t>
+          <t>Oracle Investment Proposal (as of 06/26/2026)</t>
         </is>
       </c>
     </row>
@@ -597,7 +601,7 @@
           <t>Discount %</t>
         </is>
       </c>
-      <c r="K3">
+      <c r="K3" s="9">
         <v>0.15</v>
       </c>
     </row>
@@ -658,216 +662,85 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>Discount %</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Discounted Monthly Cost</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Discounted Annual Cost</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
           <t>Custom Note</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Discount %</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Discounted Monthly Cost</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Discounted Annual Cost</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7"/>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Exadata Database Service on Cloud@Customer X11M</t>
-        </is>
-      </c>
+      <c r="B7"/>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
-      <c r="G7"/>
+      <c r="G7" s="23"/>
       <c r="H7"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Test BOM baseline: single rack; High redundancy default; license model TBD - choose BYOL or License Included.</t>
-        </is>
-      </c>
-      <c r="J7">
-        <f>$K$3</f>
-      </c>
-      <c r="K7">
-        <f>IF(G7="","",G7*(1-$K$3))</f>
-      </c>
-      <c r="L7">
-        <f>IF(K7="","",K7*12)</f>
-      </c>
+      <c r="I7" s="9">
+        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
+        <v>0.15</v>
+      </c>
+      <c r="J7" s="23">
+        <f>IF(G7="","",G7*(1-IF($K$3&gt;1,$K$3/100,$K$3)))</f>
+      </c>
+      <c r="K7" s="23">
+        <f>IF(J7="","",J7*12)</f>
+      </c>
+      <c r="L7"/>
     </row>
     <row r="8">
-      <c r="A8"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Exadata Cloud@Customer X11M Rack - single rack baseline</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8"/>
-      <c r="F8"/>
-      <c r="G8"/>
-      <c r="H8"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Each rack should be modeled as prepopulated with 2 database servers.</t>
-        </is>
-      </c>
-      <c r="J8">
-        <f>$K$3</f>
-      </c>
-      <c r="K8">
-        <f>IF(G8="","",G8*(1-$K$3))</f>
-      </c>
-      <c r="L8">
-        <f>IF(K8="","",K8*12)</f>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9"/>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Exadata Database Service on Cloud@Customer X11M - Database Server</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>2</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9"/>
-      <c r="F9"/>
-      <c r="G9"/>
-      <c r="H9"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Baseline single-rack configuration includes 2 database servers. Additional database servers increase usable memory and database cores/ECPUs.</t>
-        </is>
-      </c>
-      <c r="J9">
-        <f>$K$3</f>
-      </c>
-      <c r="K9">
-        <f>IF(G9="","",G9*(1-$K$3))</f>
-      </c>
-      <c r="L9">
-        <f>IF(K9="","",K9*12)</f>
+          <t>Monthly Total</t>
+        </is>
+      </c>
+      <c r="G8" s="23">
+        <f>SUM(G7:G7)</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="9">
+        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
+        <v>0.15</v>
+      </c>
+      <c r="J8" s="23">
+        <f>SUM(J7:J7)</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="23">
+        <f>SUM(K7:K7)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10"/>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Exadata Database Service on Cloud@Customer X11M - Storage Server</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>3</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10"/>
-      <c r="F10"/>
-      <c r="G10"/>
-      <c r="H10"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Minimum storage-server count is 3. Assumes High redundancy unless Normal redundancy is explicitly specified.</t>
-        </is>
-      </c>
-      <c r="J10">
-        <f>$K$3</f>
-      </c>
-      <c r="K10">
-        <f>IF(G10="","",G10*(1-$K$3))</f>
-      </c>
-      <c r="L10">
-        <f>IF(K10="","",K10*12)</f>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11"/>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Exadata Database ECPU - Dedicated Infrastructure</t>
-        </is>
-      </c>
-      <c r="C11"/>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11">
-        <v>744</v>
-      </c>
-      <c r="F11"/>
-      <c r="G11"/>
-      <c r="H11"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Software license model TBD - choose BYOL or License Included before final pricing.</t>
-        </is>
-      </c>
-      <c r="J11">
-        <f>$K$3</f>
-      </c>
-      <c r="K11">
-        <f>IF(G11="","",G11*(1-$K$3))</f>
-      </c>
-      <c r="L11">
-        <f>IF(K11="","",K11*12)</f>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Quote is for investment proposal only.</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Monthly Total</t>
-        </is>
-      </c>
-      <c r="G12">
-        <f>SUM(G7:G11)</f>
-      </c>
-      <c r="J12">
-        <f>$K$3</f>
-      </c>
-      <c r="K12">
-        <f>SUM(K7:K11)</f>
-      </c>
-      <c r="L12">
-        <f>SUM(L7:L11)</f>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Quote is for investment proposal only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Disclaimer: Pricing is an estimate based on Oracle Cost Estimator or user-provided list-price inputs. It is not a formal Oracle quote. Validate pricing, terms, discounts, and availability with Oracle before procurement.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:L12"/>
+  <autoFilter ref="A6:L8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add customer-facing BOM sheet
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -5,6 +5,7 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="PAAS" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Customer BOM" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -551,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -602,7 +603,7 @@
         </is>
       </c>
       <c r="K3" s="9">
-        <v>0.15</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="4">
@@ -683,7 +684,11 @@
     </row>
     <row r="7">
       <c r="A7"/>
-      <c r="B7"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Exadata Database Service on Cloud@Customer X11M</t>
+        </is>
+      </c>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
@@ -700,47 +705,484 @@
       <c r="K7" s="23">
         <f>IF(J7="","",J7*12)</f>
       </c>
-      <c r="L7"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Test BOM baseline: single rack; High redundancy default; license model TBD - choose BYOL or License Included.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
+      <c r="A8"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Monthly Total</t>
-        </is>
-      </c>
-      <c r="G8" s="23">
-        <f>SUM(G7:G7)</f>
-        <v>0</v>
-      </c>
+          <t>Exadata Cloud@Customer X11M Rack - single rack baseline</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8" s="23"/>
+      <c r="H8"/>
       <c r="I8" s="9">
         <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
         <v>0.15</v>
       </c>
       <c r="J8" s="23">
-        <f>SUM(J7:J7)</f>
+        <f>IF(G8="","",G8*(1-IF($K$3&gt;1,$K$3/100,$K$3)))</f>
+      </c>
+      <c r="K8" s="23">
+        <f>IF(J8="","",J8*12)</f>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Each rack should be modeled as prepopulated with 2 database servers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Exadata Database Service on Cloud@Customer X11M - Database Server</t>
+        </is>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9" s="23"/>
+      <c r="H9"/>
+      <c r="I9" s="9">
+        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
+        <v>0.15</v>
+      </c>
+      <c r="J9" s="23">
+        <f>IF(G9="","",G9*(1-IF($K$3&gt;1,$K$3/100,$K$3)))</f>
+      </c>
+      <c r="K9" s="23">
+        <f>IF(J9="","",J9*12)</f>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Baseline single-rack configuration includes 2 database servers. Additional database servers increase usable memory and database cores/ECPUs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Exadata Database Service on Cloud@Customer X11M - Storage Server</t>
+        </is>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10" s="23"/>
+      <c r="H10"/>
+      <c r="I10" s="9">
+        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
+        <v>0.15</v>
+      </c>
+      <c r="J10" s="23">
+        <f>IF(G10="","",G10*(1-IF($K$3&gt;1,$K$3/100,$K$3)))</f>
+      </c>
+      <c r="K10" s="23">
+        <f>IF(J10="","",J10*12)</f>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Minimum storage-server count is 3. Assumes High redundancy unless Normal redundancy is explicitly specified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Exadata Database ECPU - Dedicated Infrastructure</t>
+        </is>
+      </c>
+      <c r="C11"/>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>744</v>
+      </c>
+      <c r="F11"/>
+      <c r="G11" s="23"/>
+      <c r="H11"/>
+      <c r="I11" s="9">
+        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
+        <v>0.15</v>
+      </c>
+      <c r="J11" s="23">
+        <f>IF(G11="","",G11*(1-IF($K$3&gt;1,$K$3/100,$K$3)))</f>
+      </c>
+      <c r="K11" s="23">
+        <f>IF(J11="","",J11*12)</f>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Software license model TBD - choose BYOL or License Included before final pricing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Monthly Total</t>
+        </is>
+      </c>
+      <c r="G12" s="23">
+        <f>SUM(G7:G11)</f>
         <v>0</v>
       </c>
-      <c r="K8" s="23">
-        <f>SUM(K7:K7)</f>
+      <c r="I12" s="9">
+        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
+        <v>0.15</v>
+      </c>
+      <c r="J12" s="23">
+        <f>SUM(J7:J11)</f>
         <v>0</v>
+      </c>
+      <c r="K12" s="23">
+        <f>SUM(K7:K11)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Quote is for investment proposal only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Disclaimer: Pricing is an estimate based on Oracle Cost Estimator or user-provided list-price inputs. It is not a formal Oracle quote. Validate pricing, terms, discounts, and availability with Oracle before procurement.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:L12"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="72" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Customer BOM (as of 06/26/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Reference label: Oracle Cloud BOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Currency: USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Realm: PUBLIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>List-price customer view. Discount calculations are intentionally omitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Part Qty</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Instance Qty</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Usage Qty</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Billing Basis</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Unit List Price</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Monthly List Price</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Annual List Price</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>One-Time List Price</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Customer Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B7"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Exadata Database Service on Cloud@Customer X11M</t>
+        </is>
+      </c>
+      <c r="D7"/>
+      <c r="E7"/>
+      <c r="F7"/>
+      <c r="G7"/>
+      <c r="H7"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Test BOM baseline: single rack; High redundancy default; license model TBD - choose BYOL or License Included.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B8"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Exadata Cloud@Customer X11M Rack - single rack baseline</t>
+        </is>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Each rack should be modeled as prepopulated with 2 database servers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B9"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Exadata Database Service on Cloud@Customer X11M - Database Server</t>
+        </is>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="23"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Baseline single-rack configuration includes 2 database servers. Additional database servers increase usable memory and database cores/ECPUs.</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Quote is for investment proposal only.</t>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B10"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Exadata Database Service on Cloud@Customer X11M - Storage Server</t>
+        </is>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10"/>
+      <c r="G10"/>
+      <c r="H10"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Minimum storage-server count is 3. Assumes High redundancy unless Normal redundancy is explicitly specified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B11"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Exadata Database ECPU - Dedicated Infrastructure</t>
+        </is>
+      </c>
+      <c r="D11"/>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>744</v>
+      </c>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Software license model TBD - choose BYOL or License Included before final pricing.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Customer BOM Total</t>
+        </is>
+      </c>
+      <c r="I12" s="23">
+        <f>SUM(I7:I11)</f>
+        <v>0</v>
+      </c>
+      <c r="J12" s="23">
+        <f>SUM(J7:J11)</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="23">
+        <f>SUM(K7:K11)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Customer-facing view shows list prices only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Disclaimer: Pricing is an estimate based on Oracle Cost Estimator or user-provided list-price inputs. It is not a formal Oracle quote. Validate pricing, terms, discounts, and availability with Oracle before procurement.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:L8"/>
+  <autoFilter ref="A6:L12"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use wide environment blocks in customer BOM
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -888,21 +888,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="72" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="72" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="34" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="42" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -936,253 +938,130 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>List-price customer view. Discount calculations are intentionally omitted.</t>
+          <t>List-price customer view by environment. Discount calculations are intentionally omitted.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>Part</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Part</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Billing Basis</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Part Qty</t>
+          <t>Unit List Price</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Instance Qty</t>
+          <t>General Qty</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Usage Qty</t>
+          <t>General Hrs</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Billing Basis</t>
+          <t>General Monthly List</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Unit List Price</t>
+          <t>General Annual List</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Monthly List Price</t>
+          <t>General One-Time List</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Annual List Price</t>
+          <t>Total Qty</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>One-Time List Price</t>
+          <t>Total Monthly List</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
+          <t>Total Annual List</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Total One-Time List</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
           <t>Customer Note</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="B7"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Exadata Database Service on Cloud@Customer X11M</t>
-        </is>
-      </c>
-      <c r="D7"/>
-      <c r="E7"/>
-      <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="23"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Test BOM baseline: single rack; High redundancy default; license model TBD - choose BYOL or License Included.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="B8"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Exadata Cloud@Customer X11M Rack - single rack baseline</t>
-        </is>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8"/>
-      <c r="G8"/>
-      <c r="H8"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Each rack should be modeled as prepopulated with 2 database servers.</t>
-        </is>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>General Total</t>
+        </is>
+      </c>
+      <c r="G7" s="23">
+        <f>SUM(G7:G6)</f>
+      </c>
+      <c r="H7" s="23">
+        <f>SUM(H7:H6)</f>
+      </c>
+      <c r="I7" s="23">
+        <f>SUM(I7:I6)</f>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="B9"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Exadata Database Service on Cloud@Customer X11M - Database Server</t>
-        </is>
-      </c>
-      <c r="D9">
-        <v>2</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9"/>
-      <c r="G9"/>
-      <c r="H9"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Baseline single-rack configuration includes 2 database servers. Additional database servers increase usable memory and database cores/ECPUs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="B10"/>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Exadata Database Service on Cloud@Customer X11M - Storage Server</t>
-        </is>
-      </c>
-      <c r="D10">
-        <v>3</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10"/>
-      <c r="G10"/>
-      <c r="H10"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Minimum storage-server count is 3. Assumes High redundancy unless Normal redundancy is explicitly specified.</t>
-        </is>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>All Environments Total</t>
+        </is>
+      </c>
+      <c r="K9" s="23">
+        <f>SUM(K7:K6)</f>
+      </c>
+      <c r="L9" s="23">
+        <f>SUM(L7:L6)</f>
+      </c>
+      <c r="M9" s="23">
+        <f>SUM(M7:M6)</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="B11"/>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Exadata Database ECPU - Dedicated Infrastructure</t>
-        </is>
-      </c>
-      <c r="D11"/>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="F11">
-        <v>744</v>
-      </c>
-      <c r="G11"/>
-      <c r="H11"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="23"/>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Software license model TBD - choose BYOL or License Included before final pricing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Customer BOM Total</t>
-        </is>
-      </c>
-      <c r="I12" s="23">
-        <f>SUM(I7:I11)</f>
-        <v>0</v>
-      </c>
-      <c r="J12" s="23">
-        <f>SUM(J7:J11)</f>
-        <v>0</v>
-      </c>
-      <c r="K12" s="23">
-        <f>SUM(K7:K11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
           <t>Customer-facing view shows list prices only.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Disclaimer: Pricing is an estimate based on Oracle Cost Estimator or user-provided list-price inputs. It is not a formal Oracle quote. Validate pricing, terms, discounts, and availability with Oracle before procurement.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:L12"/>
+  <autoFilter ref="A6:N6"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify customer BOM environment totals
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -888,7 +888,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -904,7 +904,6 @@
     <col min="11" max="11" width="20" customWidth="1"/>
     <col min="12" max="12" width="20" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
-    <col min="14" max="14" width="42" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -938,130 +937,178 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>List-price customer view by environment. Discount calculations are intentionally omitted.</t>
+          <t>Environment Summary</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Monthly List</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Annual List</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>One-Time List</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B6" s="23">
+        <f>SUM(G11:G10)</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="23">
+        <f>SUM(H11:H10)</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="23">
+        <f>SUM(I11:I10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>All Environments</t>
+        </is>
+      </c>
+      <c r="B7" s="23">
+        <f>SUM(K11:K10)</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="23">
+        <f>SUM(L11:L10)</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="23">
+        <f>SUM(M11:M10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SKU Detail</t>
+        </is>
+      </c>
+      <c r="B9"/>
+      <c r="C9"/>
+      <c r="D9"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>All Environments</t>
+        </is>
+      </c>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Billing Basis</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Unit List Price</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>General Qty</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>General Hrs</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>General Monthly List</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>General Annual List</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>General One-Time List</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Hrs</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Monthly List</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Annual List</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>One-Time List</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>Total Qty</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Total Monthly List</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Total Annual List</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Total One-Time List</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Customer Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>General Total</t>
-        </is>
-      </c>
-      <c r="G7" s="23">
-        <f>SUM(G7:G6)</f>
-      </c>
-      <c r="H7" s="23">
-        <f>SUM(H7:H6)</f>
-      </c>
-      <c r="I7" s="23">
-        <f>SUM(I7:I6)</f>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>All Environments Total</t>
-        </is>
-      </c>
-      <c r="K9" s="23">
-        <f>SUM(K7:K6)</f>
-      </c>
-      <c r="L9" s="23">
-        <f>SUM(L7:L6)</f>
-      </c>
-      <c r="M9" s="23">
-        <f>SUM(M7:M6)</f>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Customer-facing view shows list prices only.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Disclaimer: Pricing is an estimate based on Oracle Cost Estimator or user-provided list-price inputs. It is not a formal Oracle quote. Validate pricing, terms, discounts, and availability with Oracle before procurement.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:N6"/>
+  <mergeCells count="3">
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="E9:I9"/>
+    <mergeCell ref="J9:M9"/>
+  </mergeCells>
+  <autoFilter ref="A10:M10"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Make customer BOM the default styled view
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -3,6 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <bookViews>
+    <workbookView activeTab="1" firstSheet="1"/>
+  </bookViews>
   <sheets>
     <sheet sheetId="1" name="PAAS" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Customer BOM" state="visible" r:id="rId5"/>
@@ -130,12 +133,60 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E2F3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF305496"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC94938"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9C918A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6D8F8D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F5D6B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6F6F6F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -150,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -205,6 +256,30 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -227,6 +302,7 @@
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
+  <!-- customerBomStyleFills -->
 </styleSheet>
 </file>
 
@@ -566,7 +642,7 @@
     <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="12" max="12" width="28" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -935,22 +1011,22 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="inlineStr" s="24">
         <is>
           <t>Environment Summary</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" t="inlineStr" s="24">
         <is>
           <t>Monthly List</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" t="inlineStr" s="24">
         <is>
           <t>Annual List</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr" s="24">
         <is>
           <t>One-Time List</t>
         </is>
@@ -995,94 +1071,94 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="inlineStr" s="25">
         <is>
           <t>SKU Detail</t>
         </is>
       </c>
-      <c r="B9"/>
-      <c r="C9"/>
-      <c r="D9"/>
-      <c r="E9" t="inlineStr">
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" t="inlineStr" s="26">
         <is>
           <t>General</t>
         </is>
       </c>
-      <c r="F9"/>
-      <c r="G9"/>
-      <c r="H9"/>
-      <c r="I9"/>
-      <c r="J9" t="inlineStr">
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" t="inlineStr" s="31">
         <is>
           <t>All Environments</t>
         </is>
       </c>
-      <c r="K9"/>
-      <c r="L9"/>
-      <c r="M9"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
+      <c r="M9" s="31"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="inlineStr" s="25">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" t="inlineStr" s="25">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" t="inlineStr" s="25">
         <is>
           <t>Billing Basis</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="inlineStr" s="25">
         <is>
           <t>Unit List Price</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" t="inlineStr" s="26">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" t="inlineStr" s="26">
         <is>
           <t>Hrs</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" t="inlineStr" s="26">
         <is>
           <t>Monthly List</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" t="inlineStr" s="26">
         <is>
           <t>Annual List</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" t="inlineStr" s="26">
         <is>
           <t>One-Time List</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" t="inlineStr" s="31">
         <is>
           <t>Total Qty</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K10" t="inlineStr" s="31">
         <is>
           <t>Total Monthly List</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L10" t="inlineStr" s="31">
         <is>
           <t>Total Annual List</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M10" t="inlineStr" s="31">
         <is>
           <t>Total One-Time List</t>
         </is>

</xml_diff>

<commit_message>
Align PAAS and customer environment layouts
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -628,21 +628,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="22" customWidth="1"/>
-    <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="28" customWidth="1" hidden="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
+    <col min="15" max="15" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -690,274 +693,185 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Service Type: PAAS</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr" s="25">
+        <is>
+          <t>SKU Detail</t>
+        </is>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" t="inlineStr" s="26">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+      <c r="K5" t="inlineStr" s="31">
+        <is>
+          <t>All Environments</t>
+        </is>
+      </c>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="inlineStr" s="25">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" t="inlineStr" s="25">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Part Qty</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Instance Qty</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Usage Qty</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Unit Price</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Monthly Cost</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Custom Label</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Discount %</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Discounted Monthly Cost</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Discounted Annual Cost</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Custom Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7"/>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Exadata Database Service on Cloud@Customer X11M</t>
-        </is>
-      </c>
-      <c r="C7"/>
-      <c r="D7"/>
-      <c r="E7"/>
-      <c r="F7"/>
-      <c r="G7" s="23"/>
-      <c r="H7"/>
-      <c r="I7" s="9">
-        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
-        <v>0.15</v>
-      </c>
-      <c r="J7" s="23">
-        <f>IF(G7="","",G7*(1-IF($K$3&gt;1,$K$3/100,$K$3)))</f>
-      </c>
-      <c r="K7" s="23">
-        <f>IF(J7="","",J7*12)</f>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Test BOM baseline: single rack; High redundancy default; license model TBD - choose BYOL or License Included.</t>
+      <c r="C6" t="inlineStr" s="25">
+        <is>
+          <t>Billing Basis</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="25">
+        <is>
+          <t>Unit List Price</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="26">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="26">
+        <is>
+          <t>Hrs</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr" s="26">
+        <is>
+          <t>List Price</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr" s="26">
+        <is>
+          <t>Disc Price</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr" s="26">
+        <is>
+          <t>One-Time List</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr" s="26">
+        <is>
+          <t>One-Time Disc</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr" s="31">
+        <is>
+          <t>Total Qty</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr" s="31">
+        <is>
+          <t>Total List Price</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr" s="31">
+        <is>
+          <t>Total Disc Price</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr" s="31">
+        <is>
+          <t>Total One-Time List</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr" s="31">
+        <is>
+          <t>Total One-Time Disc</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8"/>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Exadata Cloud@Customer X11M Rack - single rack baseline</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8"/>
-      <c r="F8"/>
-      <c r="G8" s="23"/>
-      <c r="H8"/>
-      <c r="I8" s="9">
-        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
-        <v>0.15</v>
-      </c>
-      <c r="J8" s="23">
-        <f>IF(G8="","",G8*(1-IF($K$3&gt;1,$K$3/100,$K$3)))</f>
-      </c>
-      <c r="K8" s="23">
-        <f>IF(J8="","",J8*12)</f>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Each rack should be modeled as prepopulated with 2 database servers.</t>
+      <c r="A8" t="inlineStr" s="24">
+        <is>
+          <t>Environment Summary</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9"/>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Exadata Database Service on Cloud@Customer X11M - Database Server</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>2</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9"/>
-      <c r="F9"/>
-      <c r="G9" s="23"/>
-      <c r="H9"/>
-      <c r="I9" s="9">
-        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
-        <v>0.15</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>General Total</t>
+        </is>
+      </c>
+      <c r="G9" s="23">
+        <f>SUM(G7:G6)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="23">
+        <f>SUM(H7:H6)</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="23">
+        <f>SUM(I7:I6)</f>
+        <v>0</v>
       </c>
       <c r="J9" s="23">
-        <f>IF(G9="","",G9*(1-IF($K$3&gt;1,$K$3/100,$K$3)))</f>
-      </c>
-      <c r="K9" s="23">
-        <f>IF(J9="","",J9*12)</f>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Baseline single-rack configuration includes 2 database servers. Additional database servers increase usable memory and database cores/ECPUs.</t>
-        </is>
+        <f>SUM(J7:J6)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10"/>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Exadata Database Service on Cloud@Customer X11M - Storage Server</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>3</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10"/>
-      <c r="F10"/>
-      <c r="G10" s="23"/>
-      <c r="H10"/>
-      <c r="I10" s="9">
-        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
-        <v>0.15</v>
-      </c>
-      <c r="J10" s="23">
-        <f>IF(G10="","",G10*(1-IF($K$3&gt;1,$K$3/100,$K$3)))</f>
-      </c>
-      <c r="K10" s="23">
-        <f>IF(J10="","",J10*12)</f>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Minimum storage-server count is 3. Assumes High redundancy unless Normal redundancy is explicitly specified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11"/>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Exadata Database ECPU - Dedicated Infrastructure</t>
-        </is>
-      </c>
-      <c r="C11"/>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11">
-        <v>744</v>
-      </c>
-      <c r="F11"/>
-      <c r="G11" s="23"/>
-      <c r="H11"/>
-      <c r="I11" s="9">
-        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
-        <v>0.15</v>
-      </c>
-      <c r="J11" s="23">
-        <f>IF(G11="","",G11*(1-IF($K$3&gt;1,$K$3/100,$K$3)))</f>
-      </c>
-      <c r="K11" s="23">
-        <f>IF(J11="","",J11*12)</f>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Software license model TBD - choose BYOL or License Included before final pricing.</t>
-        </is>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>All Environments Total</t>
+        </is>
+      </c>
+      <c r="L10" s="23">
+        <f>SUM(L7:L6)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="23">
+        <f>SUM(M7:M6)</f>
+        <v>0</v>
+      </c>
+      <c r="N10" s="23">
+        <f>SUM(N7:N6)</f>
+        <v>0</v>
+      </c>
+      <c r="O10" s="23">
+        <f>SUM(O7:O6)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Monthly Total</t>
-        </is>
-      </c>
-      <c r="G12" s="23">
-        <f>SUM(G7:G11)</f>
-        <v>0</v>
-      </c>
-      <c r="I12" s="9">
-        <f>IF($K$3&gt;1,$K$3/100,$K$3)</f>
-        <v>0.15</v>
-      </c>
-      <c r="J12" s="23">
-        <f>SUM(J7:J11)</f>
-        <v>0</v>
-      </c>
-      <c r="K12" s="23">
-        <f>SUM(K7:K11)</f>
-        <v>0</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Working view includes discount calculations.</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Quote is for investment proposal only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
           <t>Disclaimer: Pricing is an estimate based on Oracle Cost Estimator or user-provided list-price inputs. It is not a formal Oracle quote. Validate pricing, terms, discounts, and availability with Oracle before procurement.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:L12"/>
+  <autoFilter ref="A6:O6"/>
+  <mergeCells count="3">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="K5:O5"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1011,157 +925,124 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr" s="24">
+      <c r="A5" t="inlineStr" s="25">
+        <is>
+          <t>SKU Detail</t>
+        </is>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" t="inlineStr" s="26">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" t="inlineStr" s="31">
+        <is>
+          <t>All Environments</t>
+        </is>
+      </c>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="25">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="25">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="25">
+        <is>
+          <t>Billing Basis</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="25">
+        <is>
+          <t>Unit List Price</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="26">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="26">
+        <is>
+          <t>Hrs</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr" s="26">
+        <is>
+          <t>List Price</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr" s="26">
+        <is>
+          <t>One-Time List</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr" s="31">
+        <is>
+          <t>Total Qty</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr" s="31">
+        <is>
+          <t>Total List Price</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr" s="31">
+        <is>
+          <t>Total One-Time List</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="24">
         <is>
           <t>Environment Summary</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr" s="24">
-        <is>
-          <t>Monthly List</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr" s="24">
-        <is>
-          <t>Annual List</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr" s="24">
-        <is>
-          <t>One-Time List</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="B6" s="23">
-        <f>SUM(G11:G10)</f>
-        <v>0</v>
-      </c>
-      <c r="C6" s="23">
-        <f>SUM(H11:H10)</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="23">
-        <f>SUM(I11:I10)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>All Environments</t>
-        </is>
-      </c>
-      <c r="B7" s="23">
-        <f>SUM(K11:K10)</f>
-        <v>0</v>
-      </c>
-      <c r="C7" s="23">
-        <f>SUM(L11:L10)</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="23">
-        <f>SUM(M11:M10)</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr" s="25">
-        <is>
-          <t>SKU Detail</t>
-        </is>
-      </c>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" t="inlineStr" s="26">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26"/>
-      <c r="J9" t="inlineStr" s="31">
-        <is>
-          <t>All Environments</t>
-        </is>
-      </c>
-      <c r="K9" s="31"/>
-      <c r="L9" s="31"/>
-      <c r="M9" s="31"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>General Total</t>
+        </is>
+      </c>
+      <c r="G9" s="23">
+        <f>SUM(G7:G6)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="23">
+        <f>SUM(H7:H6)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr" s="25">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr" s="25">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr" s="25">
-        <is>
-          <t>Billing Basis</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr" s="25">
-        <is>
-          <t>Unit List Price</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr" s="26">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr" s="26">
-        <is>
-          <t>Hrs</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr" s="26">
-        <is>
-          <t>Monthly List</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr" s="26">
-        <is>
-          <t>Annual List</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr" s="26">
-        <is>
-          <t>One-Time List</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr" s="31">
-        <is>
-          <t>Total Qty</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr" s="31">
-        <is>
-          <t>Total Monthly List</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr" s="31">
-        <is>
-          <t>Total Annual List</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr" s="31">
-        <is>
-          <t>Total One-Time List</t>
-        </is>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>All Environments Total</t>
+        </is>
+      </c>
+      <c r="K10" s="23">
+        <f>SUM(K7:K6)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="23">
+        <f>SUM(L7:L6)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1179,11 +1060,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A10:M10"/>
+  <autoFilter ref="A6:M6"/>
   <mergeCells count="3">
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="E9:I9"/>
-    <mergeCell ref="J9:M9"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="J5:M5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add BOM summary, diagram, and pricing preflight
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet sheetId="1" name="PAAS" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Customer BOM" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="System Summary" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -102,7 +103,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -132,6 +133,12 @@
     <font>
       <sz val="10"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -142,7 +149,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E2F3"/>
+        <fgColor rgb="FF1F4E79"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -189,7 +196,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -197,11 +204,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -255,30 +277,34 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -651,7 +677,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Oracle Investment Proposal (as of 06/26/2026)</t>
+          <t>Oracle Investment Proposal (as of 06/27/2026)</t>
         </is>
       </c>
     </row>
@@ -806,47 +832,47 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="inlineStr" s="24">
         <is>
           <t>General Total</t>
         </is>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="32">
         <f>SUM(G7:G6)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="32">
         <f>SUM(H7:H6)</f>
         <v>0</v>
       </c>
-      <c r="I9" s="23">
+      <c r="I9" s="32">
         <f>SUM(I7:I6)</f>
         <v>0</v>
       </c>
-      <c r="J9" s="23">
+      <c r="J9" s="32">
         <f>SUM(J7:J6)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="inlineStr" s="31">
         <is>
           <t>All Environments Total</t>
         </is>
       </c>
-      <c r="L10" s="23">
+      <c r="L10" s="32">
         <f>SUM(L7:L6)</f>
         <v>0</v>
       </c>
-      <c r="M10" s="23">
+      <c r="M10" s="32">
         <f>SUM(M7:M6)</f>
         <v>0</v>
       </c>
-      <c r="N10" s="23">
+      <c r="N10" s="32">
         <f>SUM(N7:N6)</f>
         <v>0</v>
       </c>
-      <c r="O10" s="23">
+      <c r="O10" s="32">
         <f>SUM(O7:O6)</f>
         <v>0</v>
       </c>
@@ -878,7 +904,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -889,17 +915,15 @@
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
     <col min="11" max="11" width="20" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
-    <col min="13" max="13" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Customer BOM (as of 06/26/2026)</t>
+          <t>Customer BOM (as of 06/27/2026)</t>
         </is>
       </c>
     </row>
@@ -941,15 +965,13 @@
       <c r="F5" s="26"/>
       <c r="G5" s="26"/>
       <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" t="inlineStr" s="31">
+      <c r="I5" t="inlineStr" s="31">
         <is>
           <t>All Environments</t>
         </is>
       </c>
+      <c r="J5" s="31"/>
       <c r="K5" s="31"/>
-      <c r="L5" s="31"/>
-      <c r="M5" s="31"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="25">
@@ -992,17 +1014,17 @@
           <t>One-Time List</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr" s="31">
+        <is>
+          <t>Total Qty</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr" s="31">
         <is>
-          <t>Total Qty</t>
+          <t>Total List Price</t>
         </is>
       </c>
       <c r="K6" t="inlineStr" s="31">
-        <is>
-          <t>Total List Price</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr" s="31">
         <is>
           <t>Total One-Time List</t>
         </is>
@@ -1016,34 +1038,34 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="inlineStr" s="24">
         <is>
           <t>General Total</t>
         </is>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="32">
         <f>SUM(G7:G6)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="32">
         <f>SUM(H7:H6)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="inlineStr" s="31">
         <is>
           <t>All Environments Total</t>
         </is>
       </c>
-      <c r="K10" s="23">
+      <c r="J10" s="32">
+        <f>SUM(J7:J6)</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="32">
         <f>SUM(K7:K6)</f>
         <v>0</v>
       </c>
-      <c r="L10" s="23">
-        <f>SUM(L7:L6)</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1060,11 +1082,258 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:M6"/>
+  <autoFilter ref="A6:K6"/>
   <mergeCells count="3">
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="I5:K5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="88" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Configured System Summary (as of 06/27/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Reference label: Oracle Cloud BOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Source: generated from BOM rows plus Exadata X11M datasheet reference values. Pricing fields remain on PAAS and Customer BOM sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="24">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B5" s="24"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="25">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="25">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="33">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="33">
+        <is>
+          <t>Exadata Cloud@Customer X11M</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="33">
+        <is>
+          <t>Racks</t>
+        </is>
+      </c>
+      <c r="B8" s="33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="33">
+        <is>
+          <t>Database server type</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="33">
+        <is>
+          <t>X11M</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="33">
+        <is>
+          <t>Database servers</t>
+        </is>
+      </c>
+      <c r="B10" s="33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="33">
+        <is>
+          <t>Storage server type</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="33">
+        <is>
+          <t>X11M Storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="33">
+        <is>
+          <t>Storage servers</t>
+        </is>
+      </c>
+      <c r="B12" s="33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="33">
+        <is>
+          <t>Requested ECPUs</t>
+        </is>
+      </c>
+      <c r="B13" s="33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="33">
+        <is>
+          <t>Configured ECPU capacity</t>
+        </is>
+      </c>
+      <c r="B14" s="33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="33">
+        <is>
+          <t>Usable database cores</t>
+        </is>
+      </c>
+      <c r="B15" s="33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr" s="33">
+        <is>
+          <t>VM memory GB</t>
+        </is>
+      </c>
+      <c r="B16" s="33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr" s="33">
+        <is>
+          <t>Usable storage TB</t>
+        </is>
+      </c>
+      <c r="B17" s="33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr" s="33">
+        <is>
+          <t>XRMEM TB</t>
+        </is>
+      </c>
+      <c r="B18" s="33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr" s="33">
+        <is>
+          <t>Flash cache TB</t>
+        </is>
+      </c>
+      <c r="B19" s="33">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr" s="33">
+        <is>
+          <t>Max VM clusters</t>
+        </is>
+      </c>
+      <c r="B20" s="33">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr" s="33">
+        <is>
+          <t>Storage redundancy</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr" s="33">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr" s="33">
+        <is>
+          <t>License model</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr" s="33">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr" s="33">
+        <is>
+          <t>Basis / notes</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr" s="33">
+        <is>
+          <t>Cloud@Customer summary uses datasheet values; Base DB servers assumed when Base System Rack is present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Capacity values are technical sizing references, not prices. Validate server model, redundancy, local-backup assumptions, and workload requirements before procurement.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix BOM row total formulas
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -677,7 +677,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Oracle Investment Proposal (as of 06/27/2026)</t>
+          <t>Oracle Investment Proposal (as of 06/28/2026)</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="K3" s="9">
-        <v>15.0</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="4">
@@ -923,7 +923,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Customer BOM (as of 06/27/2026)</t>
+          <t>Customer BOM (as of 06/28/2026)</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Configured System Summary (as of 06/27/2026)</t>
+          <t>Configured System Summary (as of 06/28/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add BOM annual totals and Autonomous fixture
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -654,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -667,11 +667,15 @@
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
-    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="20" customWidth="1"/>
     <col min="15" max="15" width="20" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="18" max="18" width="20" customWidth="1"/>
+    <col min="19" max="19" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -684,7 +688,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Reference label: Oracle Cloud BOM</t>
+          <t>Reference label: Sample Oracle Cloud BOM</t>
         </is>
       </c>
     </row>
@@ -708,7 +712,7 @@
         </is>
       </c>
       <c r="K3" s="9">
-        <v>0.15</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="4">
@@ -737,15 +741,19 @@
       <c r="H5" s="26"/>
       <c r="I5" s="26"/>
       <c r="J5" s="26"/>
-      <c r="K5" t="inlineStr" s="31">
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" t="inlineStr" s="31">
         <is>
           <t>All Environments</t>
         </is>
       </c>
-      <c r="L5" s="31"/>
-      <c r="M5" s="31"/>
       <c r="N5" s="31"/>
       <c r="O5" s="31"/>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="31"/>
+      <c r="R5" s="31"/>
+      <c r="S5" s="31"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="25">
@@ -780,45 +788,65 @@
       </c>
       <c r="G6" t="inlineStr" s="26">
         <is>
-          <t>List Price</t>
+          <t>Monthly List</t>
         </is>
       </c>
       <c r="H6" t="inlineStr" s="26">
         <is>
-          <t>Disc Price</t>
+          <t>Annual List</t>
         </is>
       </c>
       <c r="I6" t="inlineStr" s="26">
         <is>
+          <t>Monthly Disc</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr" s="26">
+        <is>
+          <t>Annual Disc</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr" s="26">
+        <is>
           <t>One-Time List</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr" s="26">
+      <c r="L6" t="inlineStr" s="26">
         <is>
           <t>One-Time Disc</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr" s="31">
+      <c r="M6" t="inlineStr" s="31">
         <is>
           <t>Total Qty</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr" s="31">
-        <is>
-          <t>Total List Price</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr" s="31">
-        <is>
-          <t>Total Disc Price</t>
-        </is>
-      </c>
       <c r="N6" t="inlineStr" s="31">
         <is>
+          <t>Total Monthly List</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr" s="31">
+        <is>
+          <t>Total Annual List</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr" s="31">
+        <is>
+          <t>Total Monthly Disc</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr" s="31">
+        <is>
+          <t>Total Annual Disc</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr" s="31">
+        <is>
           <t>Total One-Time List</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr" s="31">
+      <c r="S6" t="inlineStr" s="31">
         <is>
           <t>Total One-Time Disc</t>
         </is>
@@ -853,6 +881,14 @@
         <f>SUM(J7:J6)</f>
         <v>0</v>
       </c>
+      <c r="K9" s="32">
+        <f>SUM(K7:K6)</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="32">
+        <f>SUM(L7:L6)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="31">
@@ -860,14 +896,6 @@
           <t>All Environments Total</t>
         </is>
       </c>
-      <c r="L10" s="32">
-        <f>SUM(L7:L6)</f>
-        <v>0</v>
-      </c>
-      <c r="M10" s="32">
-        <f>SUM(M7:M6)</f>
-        <v>0</v>
-      </c>
       <c r="N10" s="32">
         <f>SUM(N7:N6)</f>
         <v>0</v>
@@ -876,6 +904,22 @@
         <f>SUM(O7:O6)</f>
         <v>0</v>
       </c>
+      <c r="P10" s="32">
+        <f>SUM(P7:P6)</f>
+        <v>0</v>
+      </c>
+      <c r="Q10" s="32">
+        <f>SUM(Q7:Q6)</f>
+        <v>0</v>
+      </c>
+      <c r="R10" s="32">
+        <f>SUM(R7:R6)</f>
+        <v>0</v>
+      </c>
+      <c r="S10" s="32">
+        <f>SUM(S7:S6)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -892,11 +936,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:O6"/>
+  <autoFilter ref="A6:S6"/>
   <mergeCells count="3">
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="K5:O5"/>
+    <mergeCell ref="E5:L5"/>
+    <mergeCell ref="M5:S5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -904,7 +948,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -915,9 +959,11 @@
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -930,7 +976,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Reference label: Oracle Cloud BOM</t>
+          <t>Reference label: Sample Oracle Cloud BOM</t>
         </is>
       </c>
     </row>
@@ -965,13 +1011,15 @@
       <c r="F5" s="26"/>
       <c r="G5" s="26"/>
       <c r="H5" s="26"/>
-      <c r="I5" t="inlineStr" s="31">
+      <c r="I5" s="26"/>
+      <c r="J5" t="inlineStr" s="31">
         <is>
           <t>All Environments</t>
         </is>
       </c>
-      <c r="J5" s="31"/>
       <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="25">
@@ -1006,25 +1054,35 @@
       </c>
       <c r="G6" t="inlineStr" s="26">
         <is>
-          <t>List Price</t>
+          <t>Monthly List</t>
         </is>
       </c>
       <c r="H6" t="inlineStr" s="26">
         <is>
+          <t>Annual List</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr" s="26">
+        <is>
           <t>One-Time List</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr" s="31">
+      <c r="J6" t="inlineStr" s="31">
         <is>
           <t>Total Qty</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr" s="31">
-        <is>
-          <t>Total List Price</t>
-        </is>
-      </c>
       <c r="K6" t="inlineStr" s="31">
+        <is>
+          <t>Total Monthly List</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr" s="31">
+        <is>
+          <t>Total Annual List</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr" s="31">
         <is>
           <t>Total One-Time List</t>
         </is>
@@ -1051,6 +1109,10 @@
         <f>SUM(H7:H6)</f>
         <v>0</v>
       </c>
+      <c r="I9" s="32">
+        <f>SUM(I7:I6)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="31">
@@ -1058,14 +1120,18 @@
           <t>All Environments Total</t>
         </is>
       </c>
-      <c r="J10" s="32">
-        <f>SUM(J7:J6)</f>
-        <v>0</v>
-      </c>
       <c r="K10" s="32">
         <f>SUM(K7:K6)</f>
         <v>0</v>
       </c>
+      <c r="L10" s="32">
+        <f>SUM(L7:L6)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="32">
+        <f>SUM(M7:M6)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1082,11 +1148,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:K6"/>
+  <autoFilter ref="A6:M6"/>
   <mergeCells count="3">
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="J5:M5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1111,7 +1177,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Reference label: Oracle Cloud BOM</t>
+          <t>Reference label: Sample Oracle Cloud BOM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add total annual cost columns to BOM workbooks
</commit_message>
<xml_diff>
--- a/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
+++ b/oracle-cloud-bom-builder/outputs/sample-oracle-cloud-bom.xlsx
@@ -654,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S14"/>
+  <dimension ref="A1:W14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -669,26 +669,30 @@
     <col min="10" max="10" width="18" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
     <col min="14" max="14" width="20" customWidth="1"/>
-    <col min="15" max="15" width="20" customWidth="1"/>
+    <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="20" customWidth="1"/>
     <col min="17" max="17" width="20" customWidth="1"/>
     <col min="18" max="18" width="20" customWidth="1"/>
     <col min="19" max="19" width="20" customWidth="1"/>
+    <col min="20" max="20" width="20" customWidth="1"/>
+    <col min="21" max="21" width="20" customWidth="1"/>
+    <col min="22" max="22" width="20" customWidth="1"/>
+    <col min="23" max="23" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Oracle Investment Proposal (as of 06/28/2026)</t>
+          <t>Oracle Investment Proposal (as of 07/09/2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Reference label: Sample Oracle Cloud BOM</t>
+          <t>Reference label: Oracle Cloud BOM</t>
         </is>
       </c>
     </row>
@@ -712,7 +716,7 @@
         </is>
       </c>
       <c r="K3" s="9">
-        <v>15.0</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="4">
@@ -743,17 +747,21 @@
       <c r="J5" s="26"/>
       <c r="K5" s="26"/>
       <c r="L5" s="26"/>
-      <c r="M5" t="inlineStr" s="31">
+      <c r="M5" s="26"/>
+      <c r="N5" s="26"/>
+      <c r="O5" t="inlineStr" s="31">
         <is>
           <t>All Environments</t>
         </is>
       </c>
-      <c r="N5" s="31"/>
-      <c r="O5" s="31"/>
       <c r="P5" s="31"/>
       <c r="Q5" s="31"/>
       <c r="R5" s="31"/>
       <c r="S5" s="31"/>
+      <c r="T5" s="31"/>
+      <c r="U5" s="31"/>
+      <c r="V5" s="31"/>
+      <c r="W5" s="31"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="25">
@@ -816,39 +824,59 @@
           <t>One-Time Disc</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr" s="31">
+      <c r="M6" t="inlineStr" s="26">
+        <is>
+          <t>Total Annual Cost</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr" s="26">
+        <is>
+          <t>Total Annual Disc Cost</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr" s="31">
         <is>
           <t>Total Qty</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr" s="31">
+      <c r="P6" t="inlineStr" s="31">
         <is>
           <t>Total Monthly List</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr" s="31">
+      <c r="Q6" t="inlineStr" s="31">
         <is>
           <t>Total Annual List</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr" s="31">
+      <c r="R6" t="inlineStr" s="31">
         <is>
           <t>Total Monthly Disc</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr" s="31">
+      <c r="S6" t="inlineStr" s="31">
         <is>
           <t>Total Annual Disc</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr" s="31">
+      <c r="T6" t="inlineStr" s="31">
         <is>
           <t>Total One-Time List</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr" s="31">
+      <c r="U6" t="inlineStr" s="31">
         <is>
           <t>Total One-Time Disc</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr" s="31">
+        <is>
+          <t>Total Annual Cost</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr" s="31">
+        <is>
+          <t>Total Annual Disc Cost</t>
         </is>
       </c>
     </row>
@@ -889,6 +917,14 @@
         <f>SUM(L7:L6)</f>
         <v>0</v>
       </c>
+      <c r="M9" s="32">
+        <f>SUM(H9,K9)</f>
+        <v>0</v>
+      </c>
+      <c r="N9" s="32">
+        <f>SUM(J9,L9)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="31">
@@ -896,14 +932,6 @@
           <t>All Environments Total</t>
         </is>
       </c>
-      <c r="N10" s="32">
-        <f>SUM(N7:N6)</f>
-        <v>0</v>
-      </c>
-      <c r="O10" s="32">
-        <f>SUM(O7:O6)</f>
-        <v>0</v>
-      </c>
       <c r="P10" s="32">
         <f>SUM(P7:P6)</f>
         <v>0</v>
@@ -920,6 +948,22 @@
         <f>SUM(S7:S6)</f>
         <v>0</v>
       </c>
+      <c r="T10" s="32">
+        <f>SUM(T7:T6)</f>
+        <v>0</v>
+      </c>
+      <c r="U10" s="32">
+        <f>SUM(U7:U6)</f>
+        <v>0</v>
+      </c>
+      <c r="V10" s="32">
+        <f>SUM(Q10,T10)</f>
+        <v>0</v>
+      </c>
+      <c r="W10" s="32">
+        <f>SUM(S10,U10)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -936,11 +980,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:S6"/>
+  <autoFilter ref="A6:W6"/>
   <mergeCells count="3">
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:L5"/>
-    <mergeCell ref="M5:S5"/>
+    <mergeCell ref="E5:N5"/>
+    <mergeCell ref="O5:W5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -948,7 +992,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -960,23 +1004,25 @@
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="20" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
+    <col min="15" max="15" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Customer BOM (as of 06/28/2026)</t>
+          <t>Customer BOM (as of 07/09/2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Reference label: Sample Oracle Cloud BOM</t>
+          <t>Reference label: Oracle Cloud BOM</t>
         </is>
       </c>
     </row>
@@ -1012,14 +1058,16 @@
       <c r="G5" s="26"/>
       <c r="H5" s="26"/>
       <c r="I5" s="26"/>
-      <c r="J5" t="inlineStr" s="31">
+      <c r="J5" s="26"/>
+      <c r="K5" t="inlineStr" s="31">
         <is>
           <t>All Environments</t>
         </is>
       </c>
-      <c r="K5" s="31"/>
       <c r="L5" s="31"/>
       <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="25">
@@ -1067,24 +1115,34 @@
           <t>One-Time List</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr" s="31">
+      <c r="J6" t="inlineStr" s="26">
+        <is>
+          <t>Total Annual Cost</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr" s="31">
         <is>
           <t>Total Qty</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr" s="31">
+      <c r="L6" t="inlineStr" s="31">
         <is>
           <t>Total Monthly List</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr" s="31">
+      <c r="M6" t="inlineStr" s="31">
         <is>
           <t>Total Annual List</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr" s="31">
+      <c r="N6" t="inlineStr" s="31">
         <is>
           <t>Total One-Time List</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr" s="31">
+        <is>
+          <t>Total Annual Cost</t>
         </is>
       </c>
     </row>
@@ -1113,6 +1171,10 @@
         <f>SUM(I7:I6)</f>
         <v>0</v>
       </c>
+      <c r="J9" s="32">
+        <f>SUM(H9,I9)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="31">
@@ -1120,10 +1182,6 @@
           <t>All Environments Total</t>
         </is>
       </c>
-      <c r="K10" s="32">
-        <f>SUM(K7:K6)</f>
-        <v>0</v>
-      </c>
       <c r="L10" s="32">
         <f>SUM(L7:L6)</f>
         <v>0</v>
@@ -1132,6 +1190,14 @@
         <f>SUM(M7:M6)</f>
         <v>0</v>
       </c>
+      <c r="N10" s="32">
+        <f>SUM(N7:N6)</f>
+        <v>0</v>
+      </c>
+      <c r="O10" s="32">
+        <f>SUM(M10,N10)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1148,11 +1214,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:M6"/>
+  <autoFilter ref="A6:O6"/>
   <mergeCells count="3">
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="K5:O5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1170,14 +1236,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Configured System Summary (as of 06/28/2026)</t>
+          <t>Configured System Summary (as of 07/09/2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Reference label: Sample Oracle Cloud BOM</t>
+          <t>Reference label: Oracle Cloud BOM</t>
         </is>
       </c>
     </row>

</xml_diff>